<commit_message>
se modificó leerExcel, denominacionReceptor está siendo ignorado por ahora
</commit_message>
<xml_diff>
--- a/CargadorAfip/excel-datos-cargar.xlsx
+++ b/CargadorAfip/excel-datos-cargar.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Martin\Documents\repositorios\automation-AFIP\CargadorAfip\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9FC6416-CD95-4743-8F23-BE0718F3035C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2398F4C-A7CE-4CCA-87B3-A7C1B57E7F29}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="7980" xr2:uid="{84A1063F-33CD-42A6-BE24-82C3093A76E9}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12225" xr2:uid="{84A1063F-33CD-42A6-BE24-82C3093A76E9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="49">
   <si>
     <t>Mis Comprobantes Emitidos - CUIT "27927955143"</t>
   </si>
@@ -102,9 +102,6 @@
     <t>CUIT</t>
   </si>
   <si>
-    <t>asd</t>
-  </si>
-  <si>
     <t>cuenta corriente</t>
   </si>
   <si>
@@ -159,9 +156,6 @@
     <t>tora</t>
   </si>
   <si>
-    <t>Honorarios 09-2025</t>
-  </si>
-  <si>
     <t>IVA Liberado - Ley Nº 19.640</t>
   </si>
   <si>
@@ -175,6 +169,9 @@
   </si>
   <si>
     <t>Monotributista Trabajador Independiente Promovido</t>
+  </si>
+  <si>
+    <t>Honorarios 01-2026</t>
   </si>
 </sst>
 </file>
@@ -560,7 +557,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{579DA1EF-D27E-4E0B-A230-30DBFDCC0598}">
-  <dimension ref="A1:W13"/>
+  <dimension ref="A1:W14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.140625" customWidth="1"/>
@@ -571,7 +568,7 @@
     <col min="6" max="6" width="25.7109375" customWidth="1"/>
     <col min="7" max="7" width="12" customWidth="1"/>
     <col min="10" max="10" width="14.140625" customWidth="1"/>
-    <col min="11" max="11" width="22.5703125" customWidth="1"/>
+    <col min="11" max="11" width="26" customWidth="1"/>
     <col min="12" max="12" width="19.28515625" customWidth="1"/>
     <col min="13" max="13" width="59.85546875" customWidth="1"/>
     <col min="14" max="14" width="15.85546875" customWidth="1"/>
@@ -678,13 +675,13 @@
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A3" s="4">
-        <v>45987</v>
+        <v>46094</v>
       </c>
       <c r="B3" s="4">
-        <v>45987</v>
+        <v>46082</v>
       </c>
       <c r="C3" s="4">
-        <v>45987</v>
+        <v>46094</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>21</v>
@@ -707,24 +704,22 @@
       <c r="J3" s="5">
         <v>30557356254</v>
       </c>
-      <c r="K3" s="1" t="s">
+      <c r="K3" s="1"/>
+      <c r="L3" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="L3" s="5" t="s">
+      <c r="M3" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="M3" s="1" t="s">
-        <v>27</v>
-      </c>
       <c r="N3" s="1">
-        <v>15000</v>
+        <v>19000</v>
       </c>
       <c r="O3" s="6" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="P3" s="1"/>
       <c r="Q3" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="R3" s="1">
         <v>692000</v>
@@ -736,21 +731,21 @@
         <v>1</v>
       </c>
       <c r="U3" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="V3" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A4" s="4">
-        <v>45987</v>
+        <v>46094</v>
       </c>
       <c r="B4" s="4">
-        <v>45987</v>
+        <v>46082</v>
       </c>
       <c r="C4" s="4">
-        <v>45987</v>
+        <v>46094</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>21</v>
@@ -773,20 +768,18 @@
       <c r="J4" s="5">
         <v>30713647205</v>
       </c>
-      <c r="K4" s="1" t="s">
+      <c r="K4" s="1"/>
+      <c r="L4" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="L4" s="5" t="s">
+      <c r="M4" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="M4" s="1" t="s">
-        <v>27</v>
-      </c>
       <c r="N4" s="1">
-        <v>15000</v>
+        <v>19000</v>
       </c>
       <c r="O4" s="6" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="P4" s="1"/>
       <c r="Q4" s="1" t="s">
@@ -796,27 +789,27 @@
         <v>620100</v>
       </c>
       <c r="S4" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="T4" s="1">
         <v>3</v>
       </c>
       <c r="U4" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="V4" s="1" t="s">
         <v>32</v>
-      </c>
-      <c r="V4" s="1" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A5" s="4">
-        <v>45987</v>
+        <v>46094</v>
       </c>
       <c r="B5" s="4">
-        <v>45987</v>
+        <v>46082</v>
       </c>
       <c r="C5" s="4">
-        <v>45987</v>
+        <v>46094</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>21</v>
@@ -839,44 +832,42 @@
       <c r="J5" s="5">
         <v>30585060174</v>
       </c>
-      <c r="K5" s="1" t="s">
+      <c r="K5" s="1"/>
+      <c r="L5" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="L5" s="5" t="s">
+      <c r="M5" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="M5" s="1" t="s">
-        <v>27</v>
-      </c>
       <c r="N5" s="1">
-        <v>15000</v>
+        <v>19000</v>
       </c>
       <c r="O5" s="6" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="P5" s="1"/>
       <c r="Q5" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="R5" s="1"/>
       <c r="S5" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="T5" s="1"/>
       <c r="U5" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="V5" s="1"/>
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A6" s="4">
-        <v>45987</v>
+        <v>46094</v>
       </c>
       <c r="B6" s="4">
-        <v>45987</v>
+        <v>46082</v>
       </c>
       <c r="C6" s="4">
-        <v>45987</v>
+        <v>46094</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>21</v>
@@ -899,42 +890,40 @@
       <c r="J6" s="5">
         <v>30628280157</v>
       </c>
-      <c r="K6" s="1" t="s">
+      <c r="K6" s="1"/>
+      <c r="L6" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="L6" s="5" t="s">
+      <c r="M6" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="M6" s="1" t="s">
-        <v>27</v>
-      </c>
       <c r="N6" s="1">
-        <v>15000</v>
+        <v>19000</v>
       </c>
       <c r="O6" s="6" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="P6" s="1"/>
       <c r="Q6" s="1"/>
       <c r="R6" s="1"/>
       <c r="S6" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="T6" s="1"/>
       <c r="U6" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="V6" s="1"/>
     </row>
     <row r="7" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A7" s="4">
-        <v>45987</v>
+        <v>46094</v>
       </c>
       <c r="B7" s="4">
-        <v>45987</v>
+        <v>46082</v>
       </c>
       <c r="C7" s="4">
-        <v>45987</v>
+        <v>46094</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>21</v>
@@ -957,42 +946,40 @@
       <c r="J7" s="5">
         <v>30523042110</v>
       </c>
-      <c r="K7" s="1" t="s">
+      <c r="K7" s="1"/>
+      <c r="L7" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="L7" s="5" t="s">
+      <c r="M7" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="M7" s="1" t="s">
-        <v>27</v>
-      </c>
       <c r="N7" s="1">
-        <v>15000</v>
+        <v>19000</v>
       </c>
       <c r="O7" s="6" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="P7" s="1"/>
       <c r="Q7" s="1"/>
       <c r="R7" s="1"/>
       <c r="S7" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T7" s="1"/>
       <c r="U7" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="V7" s="1"/>
     </row>
     <row r="8" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A8" s="4">
-        <v>45987</v>
+        <v>46094</v>
       </c>
       <c r="B8" s="4">
-        <v>45987</v>
+        <v>46082</v>
       </c>
       <c r="C8" s="4">
-        <v>45987</v>
+        <v>46094</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>21</v>
@@ -1015,42 +1002,40 @@
       <c r="J8" s="5">
         <v>30711535353</v>
       </c>
-      <c r="K8" s="1" t="s">
+      <c r="K8" s="1"/>
+      <c r="L8" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="L8" s="5" t="s">
+      <c r="M8" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="M8" s="1" t="s">
-        <v>27</v>
-      </c>
       <c r="N8" s="1">
-        <v>15000</v>
+        <v>19000</v>
       </c>
       <c r="O8" s="6" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="P8" s="1"/>
       <c r="Q8" s="1"/>
       <c r="R8" s="1"/>
       <c r="S8" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="T8" s="1"/>
       <c r="U8" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="V8" s="1"/>
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A9" s="4">
-        <v>45987</v>
+        <v>46094</v>
       </c>
       <c r="B9" s="4">
-        <v>45987</v>
+        <v>46082</v>
       </c>
       <c r="C9" s="4">
-        <v>45987</v>
+        <v>46094</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>21</v>
@@ -1073,42 +1058,40 @@
       <c r="J9" s="5">
         <v>30707924671</v>
       </c>
-      <c r="K9" s="1" t="s">
+      <c r="K9" s="1"/>
+      <c r="L9" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="L9" s="5" t="s">
+      <c r="M9" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="M9" s="1" t="s">
-        <v>27</v>
-      </c>
       <c r="N9" s="1">
-        <v>15000</v>
+        <v>19000</v>
       </c>
       <c r="O9" s="6" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="P9" s="1"/>
       <c r="Q9" s="1"/>
       <c r="R9" s="1"/>
       <c r="S9" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T9" s="1"/>
       <c r="U9" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="V9" s="1"/>
     </row>
     <row r="10" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A10" s="4">
-        <v>45987</v>
+        <v>46094</v>
       </c>
       <c r="B10" s="4">
-        <v>45987</v>
+        <v>46082</v>
       </c>
       <c r="C10" s="4">
-        <v>45987</v>
+        <v>46094</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>21</v>
@@ -1128,57 +1111,83 @@
       <c r="I10" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J10" s="5">
-        <v>23939551689</v>
-      </c>
-      <c r="K10" s="1" t="s">
+      <c r="J10">
+        <v>30604454499</v>
+      </c>
+      <c r="K10" s="1"/>
+      <c r="L10" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="L10" s="5" t="s">
+      <c r="M10" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="M10" s="1" t="s">
-        <v>44</v>
-      </c>
       <c r="N10" s="1">
-        <v>35000</v>
-      </c>
-      <c r="O10" s="1" t="s">
-        <v>33</v>
+        <v>19000</v>
+      </c>
+      <c r="O10" s="6" t="s">
+        <v>32</v>
       </c>
       <c r="P10" s="1"/>
       <c r="Q10" s="1"/>
       <c r="R10" s="1"/>
       <c r="S10" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="T10" s="1"/>
       <c r="U10" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="V10" s="1"/>
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A11" s="4"/>
-      <c r="B11" s="4"/>
-      <c r="C11" s="4"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
-      <c r="G11" s="1"/>
-      <c r="H11" s="1"/>
-      <c r="I11" s="1"/>
-      <c r="J11" s="1"/>
+      <c r="A11" s="4">
+        <v>46094</v>
+      </c>
+      <c r="B11" s="4">
+        <v>46082</v>
+      </c>
+      <c r="C11" s="4">
+        <v>46094</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E11" s="1">
+        <v>692000</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H11" s="5">
+        <v>1</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="J11" s="5">
+        <v>23939551689</v>
+      </c>
       <c r="K11" s="1"/>
-      <c r="L11" s="1"/>
-      <c r="M11" s="1"/>
-      <c r="N11" s="1"/>
-      <c r="O11" s="1"/>
+      <c r="L11" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="M11" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="N11" s="1">
+        <v>40000</v>
+      </c>
+      <c r="O11" s="6" t="s">
+        <v>32</v>
+      </c>
       <c r="P11" s="1"/>
       <c r="Q11" s="1"/>
       <c r="R11" s="1"/>
       <c r="S11" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="T11" s="1"/>
       <c r="U11" s="1"/>
@@ -1192,11 +1201,11 @@
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
       <c r="G12" s="1"/>
-      <c r="H12" s="5"/>
+      <c r="H12" s="1"/>
       <c r="I12" s="1"/>
-      <c r="J12" s="5"/>
+      <c r="J12" s="1"/>
       <c r="K12" s="1"/>
-      <c r="L12" s="5"/>
+      <c r="L12" s="1"/>
       <c r="M12" s="1"/>
       <c r="N12" s="1"/>
       <c r="O12" s="1"/>
@@ -1204,7 +1213,7 @@
       <c r="Q12" s="1"/>
       <c r="R12" s="1"/>
       <c r="S12" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="T12" s="1"/>
       <c r="U12" s="1"/>
@@ -1230,11 +1239,32 @@
       <c r="Q13" s="1"/>
       <c r="R13" s="1"/>
       <c r="S13" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="T13" s="1"/>
       <c r="U13" s="1"/>
       <c r="V13" s="1"/>
+    </row>
+    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A14" s="4"/>
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1"/>
+      <c r="H14" s="5"/>
+      <c r="I14" s="1"/>
+      <c r="J14" s="5"/>
+      <c r="K14" s="1"/>
+      <c r="L14" s="5"/>
+      <c r="M14" s="1"/>
+      <c r="N14" s="1"/>
+      <c r="O14" s="1"/>
+      <c r="P14" s="1"/>
+      <c r="Q14" s="1"/>
+      <c r="R14" s="1"/>
+      <c r="V14" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1242,23 +1272,23 @@
     <mergeCell ref="P1:W1"/>
   </mergeCells>
   <dataValidations count="6">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D3:D10 D12:D13" xr:uid="{65122445-7F2D-4870-816C-4EEA1649DE86}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D13:D14 D3:D11" xr:uid="{65122445-7F2D-4870-816C-4EEA1649DE86}">
       <formula1>$Q$3:$Q$5</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H3:H10 H12:H13" xr:uid="{1DB658ED-94F5-475C-9F90-4396DB16B780}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H13:H14 H3:H11" xr:uid="{1DB658ED-94F5-475C-9F90-4396DB16B780}">
       <formula1>$T$3:$T$4</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="O3:O10 O12" xr:uid="{F6A4EF4E-2F44-41B9-9AD6-8E959218DA2B}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="O13 O3:O11" xr:uid="{F6A4EF4E-2F44-41B9-9AD6-8E959218DA2B}">
       <formula1>$V$3:$V$4</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F3:F10 F12:F13" xr:uid="{D8BFCFD1-DF58-4720-AF78-09A0BD018CAC}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E13:E14 R5:R13 E3:E11" xr:uid="{1C5E4F03-2A75-4D10-8058-7394FE6372AA}">
+      <formula1>$R$3:$R$4</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F13:F14 F3:F11" xr:uid="{D8BFCFD1-DF58-4720-AF78-09A0BD018CAC}">
       <formula1>$S$3:$S$13</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="L3:L10 L12:L13" xr:uid="{BBB28F2B-C955-418C-8B24-8678C25A7211}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="L13:L14 L3:L11" xr:uid="{BBB28F2B-C955-418C-8B24-8678C25A7211}">
       <formula1>$U$3:$U$10</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E3:E10 R5:R12 E12:E13" xr:uid="{1C5E4F03-2A75-4D10-8058-7394FE6372AA}">
-      <formula1>$R$3:$R$4</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Se modificó el objeto para agregar el atributo usuario, y se hizo dinámico el uso del formulario
</commit_message>
<xml_diff>
--- a/CargadorAfip/excel-datos-cargar.xlsx
+++ b/CargadorAfip/excel-datos-cargar.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Martin\Documents\repositorios\automation-AFIP\CargadorAfip\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E8134E9-4B23-4F9A-A5BF-7F978C4BD9EA}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67C30726-59D5-4575-B4B9-76ADAD4EDBE7}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12225" xr2:uid="{84A1063F-33CD-42A6-BE24-82C3093A76E9}"/>
   </bookViews>
@@ -27,9 +27,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="49">
   <si>
-    <t>Mis Comprobantes Emitidos - CUIT "27927955143"</t>
-  </si>
-  <si>
     <t>DATOS PARA COMPLETAR (NO EDITAR)</t>
   </si>
   <si>
@@ -172,6 +169,9 @@
   </si>
   <si>
     <t>Honorarios 01-2026</t>
+  </si>
+  <si>
+    <t>FERLA IZAGUIRRE MARIA LAURA</t>
   </si>
 </sst>
 </file>
@@ -580,7 +580,7 @@
   <sheetData>
     <row r="1" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>
@@ -597,7 +597,7 @@
       <c r="N1" s="7"/>
       <c r="O1" s="7"/>
       <c r="P1" s="8" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q1" s="8"/>
       <c r="R1" s="8"/>
@@ -609,68 +609,68 @@
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="H2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="I2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="J2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="K2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="L2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="M2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="N2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="N2" s="3" t="s">
+      <c r="O2" s="3" t="s">
         <v>15</v>
-      </c>
-      <c r="O2" s="3" t="s">
-        <v>16</v>
       </c>
       <c r="P2" s="1"/>
       <c r="Q2" s="3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="S2" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="S2" s="3" t="s">
+      <c r="T2" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="T2" s="3" t="s">
+      <c r="U2" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="U2" s="3" t="s">
-        <v>20</v>
-      </c>
       <c r="V2" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.25">
@@ -684,57 +684,57 @@
         <v>46094</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E3" s="1">
         <v>692000</v>
       </c>
       <c r="F3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G3" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>23</v>
       </c>
       <c r="H3" s="5">
         <v>1</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J3" s="5">
         <v>30557356254</v>
       </c>
       <c r="K3" s="1"/>
       <c r="L3" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="M3" s="1" t="s">
         <v>25</v>
-      </c>
-      <c r="M3" s="1" t="s">
-        <v>26</v>
       </c>
       <c r="N3" s="1">
         <v>19000</v>
       </c>
       <c r="O3" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="P3" s="1"/>
       <c r="Q3" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="R3" s="1">
         <v>692000</v>
       </c>
       <c r="S3" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="T3" s="1">
         <v>1</v>
       </c>
       <c r="U3" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V3" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:23" x14ac:dyDescent="0.25">
@@ -748,57 +748,57 @@
         <v>46094</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E4" s="1">
         <v>692000</v>
       </c>
       <c r="F4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G4" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>23</v>
       </c>
       <c r="H4" s="5">
         <v>1</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J4" s="5">
         <v>30713647205</v>
       </c>
       <c r="K4" s="1"/>
       <c r="L4" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="M4" s="1" t="s">
         <v>25</v>
-      </c>
-      <c r="M4" s="1" t="s">
-        <v>26</v>
       </c>
       <c r="N4" s="1">
         <v>19000</v>
       </c>
       <c r="O4" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="P4" s="1"/>
       <c r="Q4" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="R4" s="1">
         <v>620100</v>
       </c>
       <c r="S4" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="T4" s="1">
         <v>3</v>
       </c>
       <c r="U4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="V4" s="1" t="s">
         <v>31</v>
-      </c>
-      <c r="V4" s="1" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:23" x14ac:dyDescent="0.25">
@@ -812,50 +812,50 @@
         <v>46094</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E5" s="1">
         <v>692000</v>
       </c>
       <c r="F5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G5" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>23</v>
       </c>
       <c r="H5" s="5">
         <v>1</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J5" s="5">
         <v>30585060174</v>
       </c>
       <c r="K5" s="1"/>
       <c r="L5" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="M5" s="1" t="s">
         <v>25</v>
-      </c>
-      <c r="M5" s="1" t="s">
-        <v>26</v>
       </c>
       <c r="N5" s="1">
         <v>19000</v>
       </c>
       <c r="O5" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="P5" s="1"/>
       <c r="Q5" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="R5" s="1"/>
       <c r="S5" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="T5" s="1"/>
       <c r="U5" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="V5" s="1"/>
     </row>
@@ -870,48 +870,48 @@
         <v>46094</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E6" s="1">
         <v>692000</v>
       </c>
       <c r="F6" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G6" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>23</v>
       </c>
       <c r="H6" s="5">
         <v>1</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J6" s="5">
         <v>30628280157</v>
       </c>
       <c r="K6" s="1"/>
       <c r="L6" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="M6" s="1" t="s">
         <v>25</v>
-      </c>
-      <c r="M6" s="1" t="s">
-        <v>26</v>
       </c>
       <c r="N6" s="1">
         <v>19000</v>
       </c>
       <c r="O6" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="P6" s="1"/>
       <c r="Q6" s="1"/>
       <c r="R6" s="1"/>
       <c r="S6" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="T6" s="1"/>
       <c r="U6" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="V6" s="1"/>
     </row>
@@ -926,48 +926,48 @@
         <v>46094</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E7" s="1">
         <v>692000</v>
       </c>
       <c r="F7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G7" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>23</v>
       </c>
       <c r="H7" s="5">
         <v>1</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J7" s="5">
         <v>30523042110</v>
       </c>
       <c r="K7" s="1"/>
       <c r="L7" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="M7" s="1" t="s">
         <v>25</v>
-      </c>
-      <c r="M7" s="1" t="s">
-        <v>26</v>
       </c>
       <c r="N7" s="1">
         <v>19000</v>
       </c>
       <c r="O7" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="P7" s="1"/>
       <c r="Q7" s="1"/>
       <c r="R7" s="1"/>
       <c r="S7" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="T7" s="1"/>
       <c r="U7" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="V7" s="1"/>
     </row>
@@ -982,48 +982,48 @@
         <v>46094</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E8" s="1">
         <v>692000</v>
       </c>
       <c r="F8" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G8" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>23</v>
       </c>
       <c r="H8" s="5">
         <v>1</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J8" s="5">
         <v>30711535353</v>
       </c>
       <c r="K8" s="1"/>
       <c r="L8" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="M8" s="1" t="s">
         <v>25</v>
-      </c>
-      <c r="M8" s="1" t="s">
-        <v>26</v>
       </c>
       <c r="N8" s="1">
         <v>19000</v>
       </c>
       <c r="O8" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="P8" s="1"/>
       <c r="Q8" s="1"/>
       <c r="R8" s="1"/>
       <c r="S8" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="T8" s="1"/>
       <c r="U8" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="V8" s="1"/>
     </row>
@@ -1038,48 +1038,48 @@
         <v>46094</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E9" s="1">
         <v>692000</v>
       </c>
       <c r="F9" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G9" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>23</v>
       </c>
       <c r="H9" s="5">
         <v>1</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J9" s="5">
         <v>30707924671</v>
       </c>
       <c r="K9" s="1"/>
       <c r="L9" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="M9" s="1" t="s">
         <v>25</v>
-      </c>
-      <c r="M9" s="1" t="s">
-        <v>26</v>
       </c>
       <c r="N9" s="1">
         <v>19000</v>
       </c>
       <c r="O9" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="P9" s="1"/>
       <c r="Q9" s="1"/>
       <c r="R9" s="1"/>
       <c r="S9" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="T9" s="1"/>
       <c r="U9" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="V9" s="1"/>
     </row>
@@ -1094,48 +1094,48 @@
         <v>46094</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E10" s="1">
         <v>692000</v>
       </c>
       <c r="F10" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G10" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>23</v>
       </c>
       <c r="H10" s="5">
         <v>1</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J10">
         <v>30604454499</v>
       </c>
       <c r="K10" s="1"/>
       <c r="L10" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="M10" s="1" t="s">
         <v>25</v>
-      </c>
-      <c r="M10" s="1" t="s">
-        <v>26</v>
       </c>
       <c r="N10" s="1">
         <v>19000</v>
       </c>
       <c r="O10" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="P10" s="1"/>
       <c r="Q10" s="1"/>
       <c r="R10" s="1"/>
       <c r="S10" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="T10" s="1"/>
       <c r="U10" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="V10" s="1"/>
     </row>
@@ -1150,44 +1150,44 @@
         <v>46094</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E11" s="1">
         <v>692000</v>
       </c>
       <c r="F11" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G11" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>23</v>
       </c>
       <c r="H11" s="5">
         <v>1</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J11" s="5">
         <v>23939551689</v>
       </c>
       <c r="K11" s="1"/>
       <c r="L11" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M11" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N11" s="1">
         <v>40000</v>
       </c>
       <c r="O11" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="P11" s="1"/>
       <c r="Q11" s="1"/>
       <c r="R11" s="1"/>
       <c r="S11" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="T11" s="1"/>
       <c r="U11" s="1"/>
@@ -1213,7 +1213,7 @@
       <c r="Q12" s="1"/>
       <c r="R12" s="1"/>
       <c r="S12" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T12" s="1"/>
       <c r="U12" s="1"/>
@@ -1239,7 +1239,7 @@
       <c r="Q13" s="1"/>
       <c r="R13" s="1"/>
       <c r="S13" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="T13" s="1"/>
       <c r="U13" s="1"/>

</xml_diff>